<commit_message>
Fixed User Data Management System
</commit_message>
<xml_diff>
--- a/sent_log.xlsx
+++ b/sent_log.xlsx
@@ -16,14 +16,26 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="hh:mm:ss"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +58,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,168 +457,168 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>GDN Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>GDN Time</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>GDN Number</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>GDN Type</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>GRN Date</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>GRN Time</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>GRN Number</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>GRN Type</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>19:51:10</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>1234</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>EGF GDN</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>19:46:37</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>23123</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>EGF GRN -</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>12:57:15</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>FRndz GDN</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>19:50:00</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>1234</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>EGF GRN</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>13:17:29</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>FRndz GDN</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>13:30:05</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>724073</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>EGF GRN</t>
         </is>

</xml_diff>

<commit_message>
chore: ignore credentials.json and update project data
</commit_message>
<xml_diff>
--- a/sent_log.xlsx
+++ b/sent_log.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -624,6 +624,178 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>15:38:17</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>724386</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>EGF GDN</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>14:16:21</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>724423</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>EGF GRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>15:07:06</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>724292</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>EGF GRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>15:08:35</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>724365</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>EGF GRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="6" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>724405</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>EGF GRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr"/>
+      <c r="D9" s="6" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>15:12:07</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>724293</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>EGF GRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>16:23:45</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>724313</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>EGF GRN</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Optimize startup time, add Outlook send queue, enhance reconciliation column handling and update build scripts
</commit_message>
<xml_diff>
--- a/sent_log.xlsx
+++ b/sent_log.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -667,10 +667,26 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="4" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>23:51:27</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>GDN</t>
+        </is>
+      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
           <t>2026-09-01</t>
@@ -693,10 +709,26 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr"/>
-      <c r="B7" s="4" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>00:07:02</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>GDN</t>
+        </is>
+      </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
           <t>2026-09-01</t>
@@ -719,10 +751,26 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr"/>
-      <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="6" t="inlineStr"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>00:12:32</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>GDN</t>
+        </is>
+      </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
           <t>2026-09-01</t>
@@ -745,10 +793,26 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr"/>
-      <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="6" t="inlineStr"/>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>00:16:53</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>GDN</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
           <t>2026-09-01</t>
@@ -771,10 +835,22 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr"/>
-      <c r="B10" s="4" t="inlineStr"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>00:22:14</t>
+        </is>
+      </c>
       <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="6" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>FRndz GDN</t>
+        </is>
+      </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
           <t>2026-09-01</t>
@@ -793,6 +869,54 @@
       <c r="H10" s="6" t="inlineStr">
         <is>
           <t>EGF GRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr"/>
+      <c r="D11" s="6" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>00:17:04</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>GRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr"/>
+      <c r="C12" s="5" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>00:22:02</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>FRndz GRN</t>
         </is>
       </c>
     </row>

</xml_diff>